<commit_message>
Updated xlsx and pptx kda_template: correct formatting.
</commit_message>
<xml_diff>
--- a/inst/extdata/kda_template.xlsx
+++ b/inst/extdata/kda_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yougov-my.sharepoint.com/personal/emmanuel_guizar_yougov_ch/Documents/EmmanuelDrive/30-Resources/standardizedSyntaxes/YouAnalyser/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{1B88F804-6030-47C3-B0C5-FBFC17E888BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6072812B-95D2-4AB3-B4D5-915AE94AE8B6}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{1B88F804-6030-47C3-B0C5-FBFC17E888BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E9A8B3A-EBE3-4344-A44B-A7CAC4BBFF0F}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="13455" windowHeight="13170" xr2:uid="{F8C5C5B4-D325-4FB4-9D38-CF60D67FD698}"/>
+    <workbookView xWindow="58890" yWindow="-1695" windowWidth="23985" windowHeight="14655" xr2:uid="{F8C5C5B4-D325-4FB4-9D38-CF60D67FD698}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Einstellungen</t>
   </si>
@@ -121,16 +121,63 @@
   <si>
     <t>Diese Einstellungen können geändert werden</t>
   </si>
+  <si>
+    <t>Management</t>
+  </si>
+  <si>
+    <t>Team (the employees with whom you work most often)</t>
+  </si>
+  <si>
+    <t>Corporate culture</t>
+  </si>
+  <si>
+    <t>Image of Oettinger Davidoff (or an affiliated company)</t>
+  </si>
+  <si>
+    <t>Area of responsibility</t>
+  </si>
+  <si>
+    <t>Line manager</t>
+  </si>
+  <si>
+    <t>Salary (including insurance and perks)</t>
+  </si>
+  <si>
+    <t>The responsibilities assigned to me</t>
+  </si>
+  <si>
+    <t>Information and communication policy</t>
+  </si>
+  <si>
+    <t>Collaboration between departments and specialist areas</t>
+  </si>
+  <si>
+    <t>Common rooms and catering</t>
+  </si>
+  <si>
+    <t>Opportunities for further training/development</t>
+  </si>
+  <si>
+    <t>Work processes</t>
+  </si>
+  <si>
+    <t>Workload</t>
+  </si>
+  <si>
+    <t>Workstation set-up</t>
+  </si>
+  <si>
+    <t>Flexible working arrangements (e.g. part-time, working from home)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="0.000000%"/>
+    <numFmt numFmtId="166" formatCode="0.000000%"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -284,7 +331,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -330,14 +377,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -351,6 +394,7 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,6 +567,54 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>9.7994632607023596E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.5295241811895697E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.4312004231016799E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.3991414208996196E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.4907009865949106E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.2834814926873997E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.2255819031338602E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6.0890785281211599E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.8502950259500301E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.81001654830368E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.7281333937882498E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.4323658115747797E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.2517133120192697E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.9130249539741801E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.5152126983578003E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3.25106605960147E-2</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -554,7 +646,7 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.85379129129129105</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>#N/A</c:v>
@@ -575,7 +667,7 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.84834834834834805</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>#N/A</c:v>
@@ -699,6 +791,54 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>9.7994632607023596E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.5295241811895697E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.4312004231016799E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.3991414208996196E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.4907009865949106E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.2834814926873997E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.2255819031338602E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6.0890785281211599E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.8502950259500301E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.81001654830368E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.7281333937882498E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.4323658115747797E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.2517133120192697E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.9130249539741801E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.5152126983578003E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3.25106605960147E-2</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -709,22 +849,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.84009009009008995</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.87049549549549599</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.83201951951951902</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.88100600600600598</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.86054804804804796</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.86974474474474495</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>#N/A</c:v>
@@ -875,6 +1015,54 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>9.7994632607023596E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.5295241811895697E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.4312004231016799E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.3991414208996196E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.4907009865949106E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.2834814926873997E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.2255819031338602E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6.0890785281211599E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.8502950259500301E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.81001654830368E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.7281333937882498E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.4323658115747797E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.2517133120192697E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.9130249539741801E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.5152126983578003E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3.25106605960147E-2</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -903,34 +1091,34 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.73892642642642603</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.80668168168168197</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.80893393393393398</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.809309309309309</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.78509759759759801</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.80949699699699695</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.79542042042042005</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>#N/A</c:v>
+                  <c:v>0.80142642642642603</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>#N/A</c:v>
@@ -1027,6 +1215,54 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>9.7994632607023596E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.5295241811895697E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.4312004231016799E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.3991414208996196E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.4907009865949106E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.2834814926873997E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.2255819031338602E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6.0890785281211599E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.8502950259500301E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.81001654830368E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.7281333937882498E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.4323658115747797E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.2517133120192697E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.9130249539741801E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.5152126983578003E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3.25106605960147E-2</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2572,21 +2808,29 @@
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A5" s="22"/>
-      <c r="B5" s="22"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="7" t="str">
+      <c r="A5" s="22">
+        <v>13</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="30">
+        <v>9.7994632607023596E-2</v>
+      </c>
+      <c r="D5" s="24">
+        <v>0.84009009009008995</v>
+      </c>
+      <c r="E5" s="7">
         <f>IF(AND(C5="",D5=""),"",IF(AND(C5&gt;$L$8,D5&gt;$M$8),2,IF(AND(C5&gt;$L$8,D5&lt;=$M$8),4,IF(AND(C5&lt;=$L$8,D5&lt;=$M$8),3,1))))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F5" s="7" t="e">
         <f>IF($E5=1,$D5,#N/A)</f>
         <v>#N/A</v>
       </c>
-      <c r="G5" s="7" t="e">
+      <c r="G5" s="7">
         <f>IF($E5=2,$D5,#N/A)</f>
-        <v>#N/A</v>
+        <v>0.84009009009008995</v>
       </c>
       <c r="H5" s="7" t="e">
         <f>IF($E5=3,$D5,#N/A)</f>
@@ -2602,27 +2846,27 @@
       </c>
       <c r="L5" s="8">
         <f>MAX(C5:C35)</f>
-        <v>0</v>
+        <v>9.7994632607023596E-2</v>
       </c>
       <c r="M5" s="8">
         <f>MAX(D5:D35)</f>
-        <v>0</v>
-      </c>
-      <c r="O5" s="9" t="str">
+        <v>0.88100600600600598</v>
+      </c>
+      <c r="O5" s="9">
         <f t="array" ref="O5">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="P5" s="10" t="str">
         <f t="array" ref="P5">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v/>
-      </c>
-      <c r="Q5" s="9" t="str">
+        <v>The responsibilities assigned to me</v>
+      </c>
+      <c r="Q5" s="9">
         <f t="array" ref="Q5">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="R5" s="10" t="str">
         <f t="array" ref="R5">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v/>
+        <v>Management</v>
       </c>
       <c r="S5" s="9" t="str">
         <f t="array" ref="S5">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
@@ -2632,31 +2876,39 @@
         <f t="array" ref="T5">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
         <v/>
       </c>
-      <c r="U5" s="9" t="str">
+      <c r="U5" s="9">
         <f t="array" ref="U5">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="V5" s="10" t="str">
         <f t="array" ref="V5">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v/>
+        <v>Salary (including insurance and perks)</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A6" s="22"/>
-      <c r="B6" s="22"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="7" t="str">
-        <f t="shared" ref="E6:E19" si="0">IF(AND(C6="",D6=""),"",IF(AND(C6&gt;$L$8,D6&gt;$M$8),2,IF(AND(C6&gt;$L$8,D6&lt;=$M$8),4,IF(AND(C6&lt;=$L$8,D6&lt;=$M$8),3,1))))</f>
-        <v/>
+      <c r="A6" s="22">
+        <v>3</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="30">
+        <v>8.5295241811895697E-2</v>
+      </c>
+      <c r="D6" s="24">
+        <v>0.87049549549549599</v>
+      </c>
+      <c r="E6" s="7">
+        <f t="shared" ref="E6:E35" si="0">IF(AND(C6="",D6=""),"",IF(AND(C6&gt;$L$8,D6&gt;$M$8),2,IF(AND(C6&gt;$L$8,D6&lt;=$M$8),4,IF(AND(C6&lt;=$L$8,D6&lt;=$M$8),3,1))))</f>
+        <v>2</v>
       </c>
       <c r="F6" s="7" t="e">
         <f t="shared" ref="F6:F35" si="1">IF($E6=1,$D6,#N/A)</f>
         <v>#N/A</v>
       </c>
-      <c r="G6" s="7" t="e">
+      <c r="G6" s="7">
         <f t="shared" ref="G6:G35" si="2">IF($E6=2,$D6,#N/A)</f>
-        <v>#N/A</v>
+        <v>0.87049549549549599</v>
       </c>
       <c r="H6" s="7" t="e">
         <f t="shared" ref="H6:H35" si="3">IF($E6=3,$D6,#N/A)</f>
@@ -2672,27 +2924,27 @@
       </c>
       <c r="L6" s="8">
         <f>MIN(C5:C35)</f>
-        <v>0</v>
+        <v>3.25106605960147E-2</v>
       </c>
       <c r="M6" s="8">
         <f>MIN(D5:D35)</f>
-        <v>0</v>
-      </c>
-      <c r="O6" s="11" t="str">
+        <v>0.73892642642642603</v>
+      </c>
+      <c r="O6" s="11">
         <f t="array" ref="O6">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="P6" s="12" t="str">
         <f t="array" ref="P6">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v/>
-      </c>
-      <c r="Q6" s="11" t="str">
+        <v>Workstation set-up</v>
+      </c>
+      <c r="Q6" s="11">
         <f t="array" ref="Q6">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="R6" s="12" t="str">
         <f t="array" ref="R6">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v/>
+        <v>Team (the employees with whom you work most often)</v>
       </c>
       <c r="S6" s="11" t="str">
         <f t="array" ref="S6">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
@@ -2702,31 +2954,39 @@
         <f t="array" ref="T6">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
         <v/>
       </c>
-      <c r="U6" s="11" t="str">
+      <c r="U6" s="11">
         <f t="array" ref="U6">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="V6" s="12" t="str">
         <f t="array" ref="V6">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v/>
+        <v>Information and communication policy</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A7" s="22"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="7" t="str">
+      <c r="A7" s="22">
+        <v>11</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="30">
+        <v>8.4312004231016799E-2</v>
+      </c>
+      <c r="D7" s="24">
+        <v>0.83201951951951902</v>
+      </c>
+      <c r="E7" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F7" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="G7" s="7" t="e">
+      <c r="G7" s="7">
         <f t="shared" si="2"/>
-        <v>#N/A</v>
+        <v>0.83201951951951902</v>
       </c>
       <c r="H7" s="7" t="e">
         <f t="shared" si="3"/>
@@ -2754,13 +3014,13 @@
         <f t="array" ref="P7">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
         <v/>
       </c>
-      <c r="Q7" s="11" t="str">
+      <c r="Q7" s="11">
         <f t="array" ref="Q7">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="R7" s="12" t="str">
         <f t="array" ref="R7">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
-        <v/>
+        <v>Corporate culture</v>
       </c>
       <c r="S7" s="11" t="str">
         <f t="array" ref="S7">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
@@ -2770,31 +3030,39 @@
         <f t="array" ref="T7">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
         <v/>
       </c>
-      <c r="U7" s="11" t="str">
+      <c r="U7" s="11">
         <f t="array" ref="U7">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="V7" s="12" t="str">
         <f t="array" ref="V7">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
-        <v/>
+        <v>Collaboration between departments and specialist areas</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A8" s="22"/>
-      <c r="B8" s="22"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="7" t="str">
+      <c r="A8" s="22">
+        <v>12</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="30">
+        <v>8.3991414208996196E-2</v>
+      </c>
+      <c r="D8" s="24">
+        <v>0.88100600600600598</v>
+      </c>
+      <c r="E8" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F8" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="G8" s="7" t="e">
+      <c r="G8" s="7">
         <f t="shared" si="2"/>
-        <v>#N/A</v>
+        <v>0.88100600600600598</v>
       </c>
       <c r="H8" s="7" t="e">
         <f t="shared" si="3"/>
@@ -2808,13 +3076,13 @@
       <c r="K8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="L8" s="14" t="e">
+      <c r="L8" s="14">
         <f>IF(B2="Mittelwert",AVERAGE(C5:C32),MEDIAN(C5:C32))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M8" s="15" t="e">
+        <v>6.25E-2</v>
+      </c>
+      <c r="M8" s="15">
         <f>IF(B2="Mittelwert",AVERAGE(D5:D35),MEDIAN(D5:D35))</f>
-        <v>#DIV/0!</v>
+        <v>0.82570852102102099</v>
       </c>
       <c r="O8" s="11" t="str">
         <f t="array" ref="O8">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
@@ -2824,13 +3092,13 @@
         <f t="array" ref="P8">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
         <v/>
       </c>
-      <c r="Q8" s="11" t="str">
+      <c r="Q8" s="11">
         <f t="array" ref="Q8">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="R8" s="12" t="str">
         <f t="array" ref="R8">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
-        <v/>
+        <v>Image of Oettinger Davidoff (or an affiliated company)</v>
       </c>
       <c r="S8" s="11" t="str">
         <f t="array" ref="S8">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
@@ -2840,31 +3108,39 @@
         <f t="array" ref="T8">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
         <v/>
       </c>
-      <c r="U8" s="11" t="str">
+      <c r="U8" s="11">
         <f t="array" ref="U8">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="V8" s="12" t="str">
         <f t="array" ref="V8">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
-        <v/>
+        <v>Common rooms and catering</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="7" t="str">
+      <c r="A9" s="22">
+        <v>1</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="30">
+        <v>6.4907009865949106E-2</v>
+      </c>
+      <c r="D9" s="24">
+        <v>0.86054804804804796</v>
+      </c>
+      <c r="E9" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F9" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="G9" s="7" t="e">
+      <c r="G9" s="7">
         <f t="shared" si="2"/>
-        <v>#N/A</v>
+        <v>0.86054804804804796</v>
       </c>
       <c r="H9" s="7" t="e">
         <f t="shared" si="3"/>
@@ -2878,13 +3154,13 @@
       <c r="K9" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="L9" s="30">
+      <c r="L9" s="26">
         <f>ROUND(L5+L7,4)</f>
-        <v>0.01</v>
-      </c>
-      <c r="M9" s="31">
+        <v>0.108</v>
+      </c>
+      <c r="M9" s="27">
         <f>ROUND(M5+M7,4)</f>
-        <v>0.01</v>
+        <v>0.89100000000000001</v>
       </c>
       <c r="O9" s="11" t="str">
         <f t="array" ref="O9">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
@@ -2894,13 +3170,13 @@
         <f t="array" ref="P9">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
         <v/>
       </c>
-      <c r="Q9" s="11" t="str">
+      <c r="Q9" s="11">
         <f t="array" ref="Q9">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="R9" s="12" t="str">
         <f t="array" ref="R9">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
-        <v/>
+        <v>Area of responsibility</v>
       </c>
       <c r="S9" s="11" t="str">
         <f t="array" ref="S9">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
@@ -2910,31 +3186,39 @@
         <f t="array" ref="T9">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
         <v/>
       </c>
-      <c r="U9" s="11" t="str">
+      <c r="U9" s="11">
         <f t="array" ref="U9">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="V9" s="12" t="str">
         <f t="array" ref="V9">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
-        <v/>
+        <v>Opportunities for further training/development</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A10" s="22"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="7" t="str">
+      <c r="A10" s="22">
+        <v>5</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="30">
+        <v>6.2834814926873997E-2</v>
+      </c>
+      <c r="D10" s="24">
+        <v>0.86974474474474495</v>
+      </c>
+      <c r="E10" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F10" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="G10" s="7" t="e">
+      <c r="G10" s="7">
         <f t="shared" si="2"/>
-        <v>#N/A</v>
+        <v>0.86974474474474495</v>
       </c>
       <c r="H10" s="7" t="e">
         <f t="shared" si="3"/>
@@ -2948,13 +3232,13 @@
       <c r="K10" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="32">
+      <c r="L10" s="28">
         <f>ROUND(L6-L7,4)</f>
-        <v>-0.01</v>
-      </c>
-      <c r="M10" s="33">
+        <v>2.2499999999999999E-2</v>
+      </c>
+      <c r="M10" s="29">
         <f>ROUND(M6-M7,4)</f>
-        <v>-0.01</v>
+        <v>0.72889999999999999</v>
       </c>
       <c r="O10" s="11" t="str">
         <f t="array" ref="O10">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
@@ -2964,13 +3248,13 @@
         <f t="array" ref="P10">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
         <v/>
       </c>
-      <c r="Q10" s="11" t="str">
+      <c r="Q10" s="11">
         <f t="array" ref="Q10">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="R10" s="12" t="str">
         <f t="array" ref="R10">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
-        <v/>
+        <v>Line manager</v>
       </c>
       <c r="S10" s="11" t="str">
         <f t="array" ref="S10">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
@@ -2980,23 +3264,31 @@
         <f t="array" ref="T10">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
         <v/>
       </c>
-      <c r="U10" s="11" t="str">
+      <c r="U10" s="11">
         <f t="array" ref="U10">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
-        <v/>
+        <v>16</v>
       </c>
       <c r="V10" s="12" t="str">
         <f t="array" ref="V10">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
-        <v/>
+        <v>Work processes</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A11" s="22"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="7" t="str">
+      <c r="A11" s="22">
+        <v>6</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="30">
+        <v>6.2255819031338602E-2</v>
+      </c>
+      <c r="D11" s="24">
+        <v>0.73892642642642603</v>
+      </c>
+      <c r="E11" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F11" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3006,9 +3298,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H11" s="7" t="e">
+      <c r="H11" s="7">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>0.73892642642642603</v>
       </c>
       <c r="I11" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3041,27 +3333,35 @@
         <f t="array" ref="T11">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1))</f>
         <v/>
       </c>
-      <c r="U11" s="11" t="str">
+      <c r="U11" s="11">
         <f t="array" ref="U11">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="V11" s="12" t="str">
         <f t="array" ref="V11">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1))</f>
-        <v/>
+        <v>Workload</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A12" s="22"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="7" t="str">
+      <c r="A12" s="22">
+        <v>8</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="30">
+        <v>6.0890785281211599E-2</v>
+      </c>
+      <c r="D12" s="24">
+        <v>0.85379129129129105</v>
+      </c>
+      <c r="E12" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F12" s="7" t="e">
+        <v>1</v>
+      </c>
+      <c r="F12" s="7">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
+        <v>0.85379129129129105</v>
       </c>
       <c r="G12" s="7" t="e">
         <f t="shared" si="2"/>
@@ -3102,23 +3402,31 @@
         <f t="array" ref="T12">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1))</f>
         <v/>
       </c>
-      <c r="U12" s="11" t="str">
+      <c r="U12" s="11">
         <f t="array" ref="U12">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1))</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="V12" s="12" t="str">
         <f t="array" ref="V12">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1))</f>
-        <v/>
+        <v>Flexible working arrangements (e.g. part-time, working from home)</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A13" s="22"/>
-      <c r="B13" s="22"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="7" t="str">
+      <c r="A13" s="22">
+        <v>10</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="30">
+        <v>5.8502950259500301E-2</v>
+      </c>
+      <c r="D13" s="24">
+        <v>0.80668168168168197</v>
+      </c>
+      <c r="E13" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F13" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3128,9 +3436,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H13" s="7" t="e">
+      <c r="H13" s="7">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>0.80668168168168197</v>
       </c>
       <c r="I13" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3171,13 +3479,21 @@
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A14" s="22"/>
-      <c r="B14" s="22"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="7" t="str">
+      <c r="A14" s="22">
+        <v>15</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="30">
+        <v>5.81001654830368E-2</v>
+      </c>
+      <c r="D14" s="24">
+        <v>0.80893393393393398</v>
+      </c>
+      <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F14" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3187,9 +3503,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H14" s="7" t="e">
+      <c r="H14" s="7">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>0.80893393393393398</v>
       </c>
       <c r="I14" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3232,13 +3548,21 @@
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A15" s="22"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="7" t="str">
+      <c r="A15" s="22">
+        <v>14</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="30">
+        <v>5.7281333937882498E-2</v>
+      </c>
+      <c r="D15" s="24">
+        <v>0.809309309309309</v>
+      </c>
+      <c r="E15" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F15" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3248,9 +3572,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H15" s="7" t="e">
+      <c r="H15" s="7">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>0.809309309309309</v>
       </c>
       <c r="I15" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3292,13 +3616,21 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A16" s="22"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="7" t="str">
+      <c r="A16" s="22">
+        <v>9</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="30">
+        <v>5.4323658115747797E-2</v>
+      </c>
+      <c r="D16" s="24">
+        <v>0.78509759759759801</v>
+      </c>
+      <c r="E16" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F16" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3308,9 +3640,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H16" s="7" t="e">
+      <c r="H16" s="7">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>0.78509759759759801</v>
       </c>
       <c r="I16" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3350,13 +3682,21 @@
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A17" s="22"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="7" t="str">
+      <c r="A17" s="22">
+        <v>16</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="30">
+        <v>5.2517133120192697E-2</v>
+      </c>
+      <c r="D17" s="24">
+        <v>0.80949699699699695</v>
+      </c>
+      <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F17" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3366,9 +3706,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H17" s="7" t="e">
+      <c r="H17" s="7">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>0.80949699699699695</v>
       </c>
       <c r="I17" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3408,13 +3748,21 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="7" t="str">
+      <c r="A18" s="22">
+        <v>4</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="30">
+        <v>4.9130249539741801E-2</v>
+      </c>
+      <c r="D18" s="24">
+        <v>0.79542042042042005</v>
+      </c>
+      <c r="E18" s="7">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F18" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3424,9 +3772,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H18" s="7" t="e">
+      <c r="H18" s="7">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>0.79542042042042005</v>
       </c>
       <c r="I18" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3466,17 +3814,25 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A19" s="22"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="7" t="str">
+      <c r="A19" s="22">
+        <v>2</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="30">
+        <v>3.5152126983578003E-2</v>
+      </c>
+      <c r="D19" s="24">
+        <v>0.84834834834834805</v>
+      </c>
+      <c r="E19" s="7">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F19" s="7" t="e">
+        <v>1</v>
+      </c>
+      <c r="F19" s="7">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
+        <v>0.84834834834834805</v>
       </c>
       <c r="G19" s="7" t="e">
         <f t="shared" si="2"/>
@@ -3524,11 +3880,22 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A20" s="22"/>
-      <c r="B20" s="22"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="7"/>
+      <c r="A20" s="22">
+        <v>7</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="30">
+        <v>3.25106605960147E-2</v>
+      </c>
+      <c r="D20" s="24">
+        <v>0.80142642642642603</v>
+      </c>
+      <c r="E20" s="7">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
       <c r="F20" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
@@ -3537,9 +3904,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H20" s="7" t="e">
+      <c r="H20" s="7">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>0.80142642642642603</v>
       </c>
       <c r="I20" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3582,8 +3949,11 @@
       <c r="A21" s="22"/>
       <c r="B21" s="22"/>
       <c r="C21" s="23"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="7"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="F21" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
@@ -3636,10 +4006,10 @@
     <row r="22" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A22" s="22"/>
       <c r="B22" s="22"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="28"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
       <c r="E22" s="7" t="str">
-        <f t="shared" ref="E22:E35" si="5">IF(AND(C22="",D22=""),"",IF(AND(C22&gt;$L$8,D22&gt;$M$8),2,IF(AND(C22&gt;$L$8,D22&lt;=$M$8),4,IF(AND(C22&lt;=$L$8,D22&lt;=$M$8),3,1))))</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F22" s="7" t="e">
@@ -3694,10 +4064,10 @@
     <row r="23" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A23" s="22"/>
       <c r="B23" s="22"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="28"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
       <c r="E23" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F23" s="7" t="e">
@@ -3752,10 +4122,10 @@
     <row r="24" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A24" s="22"/>
       <c r="B24" s="22"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="28"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
       <c r="E24" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F24" s="7" t="e">
@@ -3810,10 +4180,10 @@
     <row r="25" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A25" s="22"/>
       <c r="B25" s="22"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="28"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
       <c r="E25" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F25" s="7" t="e">
@@ -3868,10 +4238,10 @@
     <row r="26" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A26" s="22"/>
       <c r="B26" s="22"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="28"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
       <c r="E26" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F26" s="7" t="e">
@@ -3926,10 +4296,10 @@
     <row r="27" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A27" s="22"/>
       <c r="B27" s="22"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="28"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
       <c r="E27" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F27" s="7" t="e">
@@ -3984,10 +4354,10 @@
     <row r="28" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="28"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
       <c r="E28" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F28" s="7" t="e">
@@ -4042,10 +4412,10 @@
     <row r="29" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A29" s="22"/>
       <c r="B29" s="22"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="28"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
       <c r="E29" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F29" s="7" t="e">
@@ -4100,10 +4470,10 @@
     <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30" s="22"/>
       <c r="B30" s="22"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="28"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
       <c r="E30" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F30" s="7" t="e">
@@ -4158,10 +4528,10 @@
     <row r="31" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A31" s="22"/>
       <c r="B31" s="22"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="28"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
       <c r="E31" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F31" s="7" t="e">
@@ -4216,10 +4586,10 @@
     <row r="32" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A32" s="22"/>
       <c r="B32" s="22"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="28"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
       <c r="E32" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F32" s="7" t="e">
@@ -4272,12 +4642,12 @@
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A33" s="29"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="28"/>
+      <c r="A33" s="25"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
       <c r="E33" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F33" s="7" t="e">
@@ -4330,12 +4700,12 @@
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A34" s="29"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="28"/>
+      <c r="A34" s="25"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
       <c r="E34" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F34" s="7" t="e">
@@ -4388,12 +4758,12 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A35" s="29"/>
-      <c r="B35" s="29"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="28"/>
+      <c r="A35" s="25"/>
+      <c r="B35" s="25"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
       <c r="E35" s="7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F35" s="7" t="e">

</xml_diff>

<commit_message>
Updated kda_template pptx and xlsx again to correct minor errors in formatting.
</commit_message>
<xml_diff>
--- a/inst/extdata/kda_template.xlsx
+++ b/inst/extdata/kda_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yougov-my.sharepoint.com/personal/emmanuel_guizar_yougov_ch/Documents/EmmanuelDrive/30-Resources/standardizedSyntaxes/YouAnalyser/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{1B88F804-6030-47C3-B0C5-FBFC17E888BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E9A8B3A-EBE3-4344-A44B-A7CAC4BBFF0F}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{1B88F804-6030-47C3-B0C5-FBFC17E888BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AD21E3A-56B3-437D-B2E4-0FA55AD8E3BE}"/>
   <bookViews>
-    <workbookView xWindow="58890" yWindow="-1695" windowWidth="23985" windowHeight="14655" xr2:uid="{F8C5C5B4-D325-4FB4-9D38-CF60D67FD698}"/>
+    <workbookView xWindow="34050" yWindow="-8760" windowWidth="27495" windowHeight="19020" xr2:uid="{F8C5C5B4-D325-4FB4-9D38-CF60D67FD698}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Einstellungen</t>
   </si>
@@ -120,54 +120,6 @@
   </si>
   <si>
     <t>Diese Einstellungen können geändert werden</t>
-  </si>
-  <si>
-    <t>Management</t>
-  </si>
-  <si>
-    <t>Team (the employees with whom you work most often)</t>
-  </si>
-  <si>
-    <t>Corporate culture</t>
-  </si>
-  <si>
-    <t>Image of Oettinger Davidoff (or an affiliated company)</t>
-  </si>
-  <si>
-    <t>Area of responsibility</t>
-  </si>
-  <si>
-    <t>Line manager</t>
-  </si>
-  <si>
-    <t>Salary (including insurance and perks)</t>
-  </si>
-  <si>
-    <t>The responsibilities assigned to me</t>
-  </si>
-  <si>
-    <t>Information and communication policy</t>
-  </si>
-  <si>
-    <t>Collaboration between departments and specialist areas</t>
-  </si>
-  <si>
-    <t>Common rooms and catering</t>
-  </si>
-  <si>
-    <t>Opportunities for further training/development</t>
-  </si>
-  <si>
-    <t>Work processes</t>
-  </si>
-  <si>
-    <t>Workload</t>
-  </si>
-  <si>
-    <t>Workstation set-up</t>
-  </si>
-  <si>
-    <t>Flexible working arrangements (e.g. part-time, working from home)</t>
   </si>
 </sst>
 </file>
@@ -567,54 +519,6 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="31"/>
-                <c:pt idx="0">
-                  <c:v>9.7994632607023596E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>8.5295241811895697E-2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>8.4312004231016799E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>8.3991414208996196E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>6.4907009865949106E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6.2834814926873997E-2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6.2255819031338602E-2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>6.0890785281211599E-2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>5.8502950259500301E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>5.81001654830368E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>5.7281333937882498E-2</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>5.4323658115747797E-2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>5.2517133120192697E-2</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>4.9130249539741801E-2</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>3.5152126983578003E-2</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>3.25106605960147E-2</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -646,7 +550,7 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.85379129129129105</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>#N/A</c:v>
@@ -667,7 +571,7 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.84834834834834805</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>#N/A</c:v>
@@ -791,54 +695,6 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="31"/>
-                <c:pt idx="0">
-                  <c:v>9.7994632607023596E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>8.5295241811895697E-2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>8.4312004231016799E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>8.3991414208996196E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>6.4907009865949106E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6.2834814926873997E-2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6.2255819031338602E-2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>6.0890785281211599E-2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>5.8502950259500301E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>5.81001654830368E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>5.7281333937882498E-2</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>5.4323658115747797E-2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>5.2517133120192697E-2</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>4.9130249539741801E-2</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>3.5152126983578003E-2</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>3.25106605960147E-2</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -849,22 +705,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>0.84009009009008995</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.87049549549549599</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.83201951951951902</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.88100600600600598</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.86054804804804796</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.86974474474474495</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>#N/A</c:v>
@@ -1015,54 +871,6 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="31"/>
-                <c:pt idx="0">
-                  <c:v>9.7994632607023596E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>8.5295241811895697E-2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>8.4312004231016799E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>8.3991414208996196E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>6.4907009865949106E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6.2834814926873997E-2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6.2255819031338602E-2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>6.0890785281211599E-2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>5.8502950259500301E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>5.81001654830368E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>5.7281333937882498E-2</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>5.4323658115747797E-2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>5.2517133120192697E-2</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>4.9130249539741801E-2</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>3.5152126983578003E-2</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>3.25106605960147E-2</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1091,34 +899,34 @@
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.73892642642642603</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.80668168168168197</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.80893393393393398</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.809309309309309</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.78509759759759801</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.80949699699699695</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.79542042042042005</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.80142642642642603</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>#N/A</c:v>
@@ -1215,54 +1023,6 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="31"/>
-                <c:pt idx="0">
-                  <c:v>9.7994632607023596E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>8.5295241811895697E-2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>8.4312004231016799E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>8.3991414208996196E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>6.4907009865949106E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6.2834814926873997E-2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6.2255819031338602E-2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>6.0890785281211599E-2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>5.8502950259500301E-2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>5.81001654830368E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>5.7281333937882498E-2</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>5.4323658115747797E-2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>5.2517133120192697E-2</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>4.9130249539741801E-2</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>3.5152126983578003E-2</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>3.25106605960147E-2</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2808,29 +2568,21 @@
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A5" s="22">
-        <v>13</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="30">
-        <v>9.7994632607023596E-2</v>
-      </c>
-      <c r="D5" s="24">
-        <v>0.84009009009008995</v>
-      </c>
-      <c r="E5" s="7">
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="7" t="str">
         <f>IF(AND(C5="",D5=""),"",IF(AND(C5&gt;$L$8,D5&gt;$M$8),2,IF(AND(C5&gt;$L$8,D5&lt;=$M$8),4,IF(AND(C5&lt;=$L$8,D5&lt;=$M$8),3,1))))</f>
-        <v>2</v>
+        <v/>
       </c>
       <c r="F5" s="7" t="e">
         <f>IF($E5=1,$D5,#N/A)</f>
         <v>#N/A</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="7" t="e">
         <f>IF($E5=2,$D5,#N/A)</f>
-        <v>0.84009009009008995</v>
+        <v>#N/A</v>
       </c>
       <c r="H5" s="7" t="e">
         <f>IF($E5=3,$D5,#N/A)</f>
@@ -2846,27 +2598,27 @@
       </c>
       <c r="L5" s="8">
         <f>MAX(C5:C35)</f>
-        <v>9.7994632607023596E-2</v>
+        <v>0</v>
       </c>
       <c r="M5" s="8">
         <f>MAX(D5:D35)</f>
-        <v>0.88100600600600598</v>
-      </c>
-      <c r="O5" s="9">
+        <v>0</v>
+      </c>
+      <c r="O5" s="9" t="str">
         <f t="array" ref="O5">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v>8</v>
+        <v/>
       </c>
       <c r="P5" s="10" t="str">
         <f t="array" ref="P5">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v>The responsibilities assigned to me</v>
-      </c>
-      <c r="Q5" s="9">
+        <v/>
+      </c>
+      <c r="Q5" s="9" t="str">
         <f t="array" ref="Q5">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v>13</v>
+        <v/>
       </c>
       <c r="R5" s="10" t="str">
         <f t="array" ref="R5">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v>Management</v>
+        <v/>
       </c>
       <c r="S5" s="9" t="str">
         <f t="array" ref="S5">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
@@ -2876,39 +2628,31 @@
         <f t="array" ref="T5">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
         <v/>
       </c>
-      <c r="U5" s="9">
+      <c r="U5" s="9" t="str">
         <f t="array" ref="U5">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v>6</v>
+        <v/>
       </c>
       <c r="V5" s="10" t="str">
         <f t="array" ref="V5">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(1:1)),1))</f>
-        <v>Salary (including insurance and perks)</v>
+        <v/>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A6" s="22">
-        <v>3</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="30">
-        <v>8.5295241811895697E-2</v>
-      </c>
-      <c r="D6" s="24">
-        <v>0.87049549549549599</v>
-      </c>
-      <c r="E6" s="7">
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="7" t="str">
         <f t="shared" ref="E6:E35" si="0">IF(AND(C6="",D6=""),"",IF(AND(C6&gt;$L$8,D6&gt;$M$8),2,IF(AND(C6&gt;$L$8,D6&lt;=$M$8),4,IF(AND(C6&lt;=$L$8,D6&lt;=$M$8),3,1))))</f>
-        <v>2</v>
+        <v/>
       </c>
       <c r="F6" s="7" t="e">
         <f t="shared" ref="F6:F35" si="1">IF($E6=1,$D6,#N/A)</f>
         <v>#N/A</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="7" t="e">
         <f t="shared" ref="G6:G35" si="2">IF($E6=2,$D6,#N/A)</f>
-        <v>0.87049549549549599</v>
+        <v>#N/A</v>
       </c>
       <c r="H6" s="7" t="e">
         <f t="shared" ref="H6:H35" si="3">IF($E6=3,$D6,#N/A)</f>
@@ -2924,27 +2668,27 @@
       </c>
       <c r="L6" s="8">
         <f>MIN(C5:C35)</f>
-        <v>3.25106605960147E-2</v>
+        <v>0</v>
       </c>
       <c r="M6" s="8">
         <f>MIN(D5:D35)</f>
-        <v>0.73892642642642603</v>
-      </c>
-      <c r="O6" s="11">
+        <v>0</v>
+      </c>
+      <c r="O6" s="11" t="str">
         <f t="array" ref="O6">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v>2</v>
+        <v/>
       </c>
       <c r="P6" s="12" t="str">
         <f t="array" ref="P6">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v>Workstation set-up</v>
-      </c>
-      <c r="Q6" s="11">
+        <v/>
+      </c>
+      <c r="Q6" s="11" t="str">
         <f t="array" ref="Q6">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v>3</v>
+        <v/>
       </c>
       <c r="R6" s="12" t="str">
         <f t="array" ref="R6">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v>Team (the employees with whom you work most often)</v>
+        <v/>
       </c>
       <c r="S6" s="11" t="str">
         <f t="array" ref="S6">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
@@ -2954,39 +2698,31 @@
         <f t="array" ref="T6">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
         <v/>
       </c>
-      <c r="U6" s="11">
+      <c r="U6" s="11" t="str">
         <f t="array" ref="U6">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v>10</v>
+        <v/>
       </c>
       <c r="V6" s="12" t="str">
         <f t="array" ref="V6">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(2:2)),1))</f>
-        <v>Information and communication policy</v>
+        <v/>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A7" s="22">
-        <v>11</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="30">
-        <v>8.4312004231016799E-2</v>
-      </c>
-      <c r="D7" s="24">
-        <v>0.83201951951951902</v>
-      </c>
-      <c r="E7" s="7">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v/>
       </c>
       <c r="F7" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.83201951951951902</v>
+        <v>#N/A</v>
       </c>
       <c r="H7" s="7" t="e">
         <f t="shared" si="3"/>
@@ -3014,13 +2750,13 @@
         <f t="array" ref="P7">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
         <v/>
       </c>
-      <c r="Q7" s="11">
+      <c r="Q7" s="11" t="str">
         <f t="array" ref="Q7">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
-        <v>11</v>
+        <v/>
       </c>
       <c r="R7" s="12" t="str">
         <f t="array" ref="R7">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
-        <v>Corporate culture</v>
+        <v/>
       </c>
       <c r="S7" s="11" t="str">
         <f t="array" ref="S7">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
@@ -3030,39 +2766,31 @@
         <f t="array" ref="T7">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
         <v/>
       </c>
-      <c r="U7" s="11">
+      <c r="U7" s="11" t="str">
         <f t="array" ref="U7">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
-        <v>15</v>
+        <v/>
       </c>
       <c r="V7" s="12" t="str">
         <f t="array" ref="V7">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(3:3)),1))</f>
-        <v>Collaboration between departments and specialist areas</v>
+        <v/>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A8" s="22">
-        <v>12</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="30">
-        <v>8.3991414208996196E-2</v>
-      </c>
-      <c r="D8" s="24">
-        <v>0.88100600600600598</v>
-      </c>
-      <c r="E8" s="7">
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v/>
       </c>
       <c r="F8" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.88100600600600598</v>
+        <v>#N/A</v>
       </c>
       <c r="H8" s="7" t="e">
         <f t="shared" si="3"/>
@@ -3076,13 +2804,13 @@
       <c r="K8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="L8" s="14">
+      <c r="L8" s="14" t="e">
         <f>IF(B2="Mittelwert",AVERAGE(C5:C32),MEDIAN(C5:C32))</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="M8" s="15">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M8" s="15" t="e">
         <f>IF(B2="Mittelwert",AVERAGE(D5:D35),MEDIAN(D5:D35))</f>
-        <v>0.82570852102102099</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="O8" s="11" t="str">
         <f t="array" ref="O8">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
@@ -3092,13 +2820,13 @@
         <f t="array" ref="P8">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
         <v/>
       </c>
-      <c r="Q8" s="11">
+      <c r="Q8" s="11" t="str">
         <f t="array" ref="Q8">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
-        <v>12</v>
+        <v/>
       </c>
       <c r="R8" s="12" t="str">
         <f t="array" ref="R8">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
-        <v>Image of Oettinger Davidoff (or an affiliated company)</v>
+        <v/>
       </c>
       <c r="S8" s="11" t="str">
         <f t="array" ref="S8">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
@@ -3108,39 +2836,31 @@
         <f t="array" ref="T8">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
         <v/>
       </c>
-      <c r="U8" s="11">
+      <c r="U8" s="11" t="str">
         <f t="array" ref="U8">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
-        <v>14</v>
+        <v/>
       </c>
       <c r="V8" s="12" t="str">
         <f t="array" ref="V8">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(4:4)),1))</f>
-        <v>Common rooms and catering</v>
+        <v/>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A9" s="22">
-        <v>1</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="30">
-        <v>6.4907009865949106E-2</v>
-      </c>
-      <c r="D9" s="24">
-        <v>0.86054804804804796</v>
-      </c>
-      <c r="E9" s="7">
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v/>
       </c>
       <c r="F9" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.86054804804804796</v>
+        <v>#N/A</v>
       </c>
       <c r="H9" s="7" t="e">
         <f t="shared" si="3"/>
@@ -3156,11 +2876,11 @@
       </c>
       <c r="L9" s="26">
         <f>ROUND(L5+L7,4)</f>
-        <v>0.108</v>
+        <v>0.01</v>
       </c>
       <c r="M9" s="27">
         <f>ROUND(M5+M7,4)</f>
-        <v>0.89100000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="O9" s="11" t="str">
         <f t="array" ref="O9">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
@@ -3170,13 +2890,13 @@
         <f t="array" ref="P9">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
         <v/>
       </c>
-      <c r="Q9" s="11">
+      <c r="Q9" s="11" t="str">
         <f t="array" ref="Q9">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
-        <v>1</v>
+        <v/>
       </c>
       <c r="R9" s="12" t="str">
         <f t="array" ref="R9">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
-        <v>Area of responsibility</v>
+        <v/>
       </c>
       <c r="S9" s="11" t="str">
         <f t="array" ref="S9">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
@@ -3186,39 +2906,31 @@
         <f t="array" ref="T9">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
         <v/>
       </c>
-      <c r="U9" s="11">
+      <c r="U9" s="11" t="str">
         <f t="array" ref="U9">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
-        <v>9</v>
+        <v/>
       </c>
       <c r="V9" s="12" t="str">
         <f t="array" ref="V9">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(5:5)),1))</f>
-        <v>Opportunities for further training/development</v>
+        <v/>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A10" s="22">
-        <v>5</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="30">
-        <v>6.2834814926873997E-2</v>
-      </c>
-      <c r="D10" s="24">
-        <v>0.86974474474474495</v>
-      </c>
-      <c r="E10" s="7">
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v/>
       </c>
       <c r="F10" s="7" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="7" t="e">
         <f t="shared" si="2"/>
-        <v>0.86974474474474495</v>
+        <v>#N/A</v>
       </c>
       <c r="H10" s="7" t="e">
         <f t="shared" si="3"/>
@@ -3234,11 +2946,11 @@
       </c>
       <c r="L10" s="28">
         <f>ROUND(L6-L7,4)</f>
-        <v>2.2499999999999999E-2</v>
+        <v>-0.01</v>
       </c>
       <c r="M10" s="29">
         <f>ROUND(M6-M7,4)</f>
-        <v>0.72889999999999999</v>
+        <v>-0.01</v>
       </c>
       <c r="O10" s="11" t="str">
         <f t="array" ref="O10">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
@@ -3248,13 +2960,13 @@
         <f t="array" ref="P10">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=P$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
         <v/>
       </c>
-      <c r="Q10" s="11">
+      <c r="Q10" s="11" t="str">
         <f t="array" ref="Q10">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
-        <v>5</v>
+        <v/>
       </c>
       <c r="R10" s="12" t="str">
         <f t="array" ref="R10">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=R$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
-        <v>Line manager</v>
+        <v/>
       </c>
       <c r="S10" s="11" t="str">
         <f t="array" ref="S10">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
@@ -3264,31 +2976,23 @@
         <f t="array" ref="T10">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
         <v/>
       </c>
-      <c r="U10" s="11">
+      <c r="U10" s="11" t="str">
         <f t="array" ref="U10">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
-        <v>16</v>
+        <v/>
       </c>
       <c r="V10" s="12" t="str">
         <f t="array" ref="V10">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(6:6)),1))</f>
-        <v>Work processes</v>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A11" s="22">
-        <v>6</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="30">
-        <v>6.2255819031338602E-2</v>
-      </c>
-      <c r="D11" s="24">
-        <v>0.73892642642642603</v>
-      </c>
-      <c r="E11" s="7">
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F11" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3298,9 +3002,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="7" t="e">
         <f t="shared" si="3"/>
-        <v>0.73892642642642603</v>
+        <v>#N/A</v>
       </c>
       <c r="I11" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3333,35 +3037,27 @@
         <f t="array" ref="T11">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1))</f>
         <v/>
       </c>
-      <c r="U11" s="11">
+      <c r="U11" s="11" t="str">
         <f t="array" ref="U11">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1))</f>
-        <v>4</v>
+        <v/>
       </c>
       <c r="V11" s="12" t="str">
         <f t="array" ref="V11">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(7:7)),1))</f>
-        <v>Workload</v>
+        <v/>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A12" s="22">
-        <v>8</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="30">
-        <v>6.0890785281211599E-2</v>
-      </c>
-      <c r="D12" s="24">
-        <v>0.85379129129129105</v>
-      </c>
-      <c r="E12" s="7">
+      <c r="A12" s="22"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="F12" s="7">
+        <v/>
+      </c>
+      <c r="F12" s="7" t="e">
         <f t="shared" si="1"/>
-        <v>0.85379129129129105</v>
+        <v>#N/A</v>
       </c>
       <c r="G12" s="7" t="e">
         <f t="shared" si="2"/>
@@ -3402,31 +3098,23 @@
         <f t="array" ref="T12">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=T$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1))</f>
         <v/>
       </c>
-      <c r="U12" s="11">
+      <c r="U12" s="11" t="str">
         <f t="array" ref="U12">IF(ISERROR(INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1)),"",INDEX($A$5:$A$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1))</f>
-        <v>7</v>
+        <v/>
       </c>
       <c r="V12" s="12" t="str">
         <f t="array" ref="V12">IF(ISERROR(INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1)),"",INDEX($B$5:$B$35,SMALL(IF($E$5:$E$35=V$4,ROW($E$5:$E$35)-4,""),ROW(8:8)),1))</f>
-        <v>Flexible working arrangements (e.g. part-time, working from home)</v>
+        <v/>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A13" s="22">
-        <v>10</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="30">
-        <v>5.8502950259500301E-2</v>
-      </c>
-      <c r="D13" s="24">
-        <v>0.80668168168168197</v>
-      </c>
-      <c r="E13" s="7">
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F13" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3436,9 +3124,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="7" t="e">
         <f t="shared" si="3"/>
-        <v>0.80668168168168197</v>
+        <v>#N/A</v>
       </c>
       <c r="I13" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3479,21 +3167,13 @@
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A14" s="22">
-        <v>15</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="30">
-        <v>5.81001654830368E-2</v>
-      </c>
-      <c r="D14" s="24">
-        <v>0.80893393393393398</v>
-      </c>
-      <c r="E14" s="7">
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F14" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3503,9 +3183,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="7" t="e">
         <f t="shared" si="3"/>
-        <v>0.80893393393393398</v>
+        <v>#N/A</v>
       </c>
       <c r="I14" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3548,21 +3228,13 @@
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A15" s="22">
-        <v>14</v>
-      </c>
-      <c r="B15" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="30">
-        <v>5.7281333937882498E-2</v>
-      </c>
-      <c r="D15" s="24">
-        <v>0.809309309309309</v>
-      </c>
-      <c r="E15" s="7">
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F15" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3572,9 +3244,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="7" t="e">
         <f t="shared" si="3"/>
-        <v>0.809309309309309</v>
+        <v>#N/A</v>
       </c>
       <c r="I15" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3616,21 +3288,13 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A16" s="22">
-        <v>9</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" s="30">
-        <v>5.4323658115747797E-2</v>
-      </c>
-      <c r="D16" s="24">
-        <v>0.78509759759759801</v>
-      </c>
-      <c r="E16" s="7">
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F16" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3640,9 +3304,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="7" t="e">
         <f t="shared" si="3"/>
-        <v>0.78509759759759801</v>
+        <v>#N/A</v>
       </c>
       <c r="I16" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3682,21 +3346,13 @@
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A17" s="22">
-        <v>16</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" s="30">
-        <v>5.2517133120192697E-2</v>
-      </c>
-      <c r="D17" s="24">
-        <v>0.80949699699699695</v>
-      </c>
-      <c r="E17" s="7">
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F17" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3706,9 +3362,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="7" t="e">
         <f t="shared" si="3"/>
-        <v>0.80949699699699695</v>
+        <v>#N/A</v>
       </c>
       <c r="I17" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3748,21 +3404,13 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A18" s="22">
-        <v>4</v>
-      </c>
-      <c r="B18" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" s="30">
-        <v>4.9130249539741801E-2</v>
-      </c>
-      <c r="D18" s="24">
-        <v>0.79542042042042005</v>
-      </c>
-      <c r="E18" s="7">
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F18" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3772,9 +3420,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="7" t="e">
         <f t="shared" si="3"/>
-        <v>0.79542042042042005</v>
+        <v>#N/A</v>
       </c>
       <c r="I18" s="7" t="e">
         <f t="shared" si="4"/>
@@ -3814,25 +3462,17 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A19" s="22">
-        <v>2</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="C19" s="30">
-        <v>3.5152126983578003E-2</v>
-      </c>
-      <c r="D19" s="24">
-        <v>0.84834834834834805</v>
-      </c>
-      <c r="E19" s="7">
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="F19" s="7">
+        <v/>
+      </c>
+      <c r="F19" s="7" t="e">
         <f t="shared" si="1"/>
-        <v>0.84834834834834805</v>
+        <v>#N/A</v>
       </c>
       <c r="G19" s="7" t="e">
         <f t="shared" si="2"/>
@@ -3880,21 +3520,13 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A20" s="22">
-        <v>7</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" s="30">
-        <v>3.25106605960147E-2</v>
-      </c>
-      <c r="D20" s="24">
-        <v>0.80142642642642603</v>
-      </c>
-      <c r="E20" s="7">
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="F20" s="7" t="e">
         <f t="shared" si="1"/>
@@ -3904,9 +3536,9 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="7" t="e">
         <f t="shared" si="3"/>
-        <v>0.80142642642642603</v>
+        <v>#N/A</v>
       </c>
       <c r="I20" s="7" t="e">
         <f t="shared" si="4"/>

</xml_diff>